<commit_message>
Week 7 9:30 window: red-team pulls and downgrades applied across thesis families, 23 PLAY
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DRV9GgxaEbuX9GLrrgpBnz
</commit_message>
<xml_diff>
--- a/docs/weekly/SLATE_FULL_2026_W07.xlsx
+++ b/docs/weekly/SLATE_FULL_2026_W07.xlsx
@@ -486,7 +486,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Inputs used (UTC). ESPN game-summary Outs (5 names per team cap, not the official inactives): 2026-10-25T12:01:29Z. Sleeper status overlay (newer Out replaces the NFL row): 2026-10-25T12:01:26+00:00. nflverse depth charts: 2026-10-25T06:01:49Z; nflverse injuries: no timestamp in the feed. Lines: ESPN/DraftKings fetched 2026-10-25T12:10Z (no prices; the per-line last_updated_utc stamps run ahead of the fetch time and their zone is unverified, so no recency claim is made from them). Official inactives: not used (the ESPN feed carries injuries, not the NFL inactive list). Code: git c21ee9a.</t>
+          <t>Inputs used (UTC). ESPN game-summary Outs (5 names per team cap, not the official inactives): 2026-10-25T12:01:29Z. Sleeper status overlay (newer Out replaces the NFL row): 2026-10-25T12:01:26+00:00. nflverse depth charts: 2026-10-25T06:01:49Z; nflverse injuries: no timestamp in the feed. Lines: ESPN/DraftKings fetched 2026-10-25T12:10Z (no prices; the per-line last_updated_utc stamps run ahead of the fetch time and their zone is unverified, so no recency claim is made from them). Official inactives: not used (the ESPN feed carries injuries, not the NFL inactive list). Code: git 1cd37ed.</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
@@ -700,58 +700,58 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>NYG@HOU: Woody Marks anytime TD + GB@DET: Jordan Love pass TD 1+</t>
+          <t>IND@MIN: Kyler Murray rush_yds U26.5 + GB@DET: Jordan Love pass TD 2+</t>
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>0.3720000000000001</v>
+        <v>0.37</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>0.51</v>
+        <v>0.507</v>
       </c>
       <c r="D15" t="n">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="E15" t="n">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>NYG@HOU: Woody Marks anytime TD + LA@LV: Matthew Stafford pass TD 1+</t>
+          <t>CIN@BAL: Chase Brown rush_att O11.5 + GB@DET: Jordan Love pass TD 2+</t>
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>0.371</v>
+        <v>0.369</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>0.509</v>
+        <v>0.507</v>
       </c>
       <c r="D16" t="n">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="E16" t="n">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>NYG@HOU: Woody Marks anytime TD + SF@ATL: Brock Purdy pass TD 1+</t>
+          <t>SF@ATL: George Kittle anytime TD + GB@DET: Jordan Love pass TD 1+</t>
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>0.371</v>
+        <v>0.36</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>0.507</v>
+        <v>0.478</v>
       </c>
       <c r="D17" t="n">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="E17" t="n">
-        <v>202</v>
+        <v>212</v>
       </c>
     </row>
     <row r="18"/>
@@ -948,39 +948,39 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>NYG@HOU: Woody Marks rec U2.5 + SF@ATL: George Kittle anytime TD + SF@ATL: Brock Purdy pass TD 1+</t>
+          <t>DEN@ARI: Tyler Allgeier rec U2.5 + SF@ATL: George Kittle anytime TD + SF@ATL: Brock Purdy pass TD 1+</t>
         </is>
       </c>
       <c r="B31" s="6" t="n">
-        <v>0.266</v>
+        <v>0.259</v>
       </c>
       <c r="C31" s="6" t="n">
-        <v>0.433</v>
+        <v>0.416</v>
       </c>
       <c r="D31" t="n">
-        <v>276</v>
+        <v>286</v>
       </c>
       <c r="E31" t="n">
-        <v>322</v>
+        <v>333</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>DAL@PHI: Javonte Williams rush_att U16.5 + SF@ATL: George Kittle anytime TD + SF@ATL: Brock Purdy pass TD 1+</t>
+          <t>NYG@HOU: Xavier Hutchinson rec O1.5 + SF@ATL: George Kittle anytime TD + SF@ATL: Brock Purdy pass TD 1+</t>
         </is>
       </c>
       <c r="B32" s="6" t="n">
-        <v>0.261</v>
+        <v>0.258</v>
       </c>
       <c r="C32" s="6" t="n">
-        <v>0.421</v>
+        <v>0.414</v>
       </c>
       <c r="D32" t="n">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="E32" t="n">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
     <row r="33"/>
@@ -1028,77 +1028,77 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>IND@MIN: Kyler Murray rush_yds U26.5 + CIN@BAL: Chase Brown rush_att O11.5 + NYG@HOU: Woody Marks rec U2.5 + GB@DET: Jordan Love pass TD 1+</t>
+          <t>IND@MIN: Kyler Murray rush_yds U26.5 + CIN@BAL: Chase Brown rush_att O11.5 + DEN@ARI: Tyler Allgeier rec U2.5 + GB@DET: Jordan Love pass TD 1+</t>
         </is>
       </c>
       <c r="B37" s="6" t="n">
-        <v>0.197</v>
+        <v>0.192</v>
       </c>
       <c r="C37" s="6" t="n">
-        <v>0.479</v>
+        <v>0.459</v>
       </c>
       <c r="D37" t="n">
-        <v>408</v>
+        <v>422</v>
       </c>
       <c r="E37" t="n">
-        <v>469</v>
+        <v>484</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>IND@MIN: Kyler Murray rush_yds U26.5 + CIN@BAL: Chase Brown rush_att O11.5 + NYG@HOU: Woody Marks rec U2.5 + LA@LV: Matthew Stafford pass TD 1+</t>
+          <t>IND@MIN: Kyler Murray rush_yds U26.5 + CIN@BAL: Chase Brown rush_att O11.5 + DEN@ARI: Tyler Allgeier rec U2.5 + LA@LV: Matthew Stafford pass TD 1+</t>
         </is>
       </c>
       <c r="B38" s="6" t="n">
-        <v>0.196</v>
+        <v>0.191</v>
       </c>
       <c r="C38" s="6" t="n">
-        <v>0.478</v>
+        <v>0.458</v>
       </c>
       <c r="D38" t="n">
-        <v>409</v>
+        <v>422</v>
       </c>
       <c r="E38" t="n">
-        <v>470</v>
+        <v>485</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>IND@MIN: Kyler Murray rush_yds U26.5 + CIN@BAL: Chase Brown rush_att O11.5 + NYG@HOU: Woody Marks rec U2.5 + SF@ATL: Brock Purdy pass TD 1+</t>
+          <t>IND@MIN: Kyler Murray rush_yds U26.5 + CIN@BAL: Chase Brown rush_att O11.5 + NYG@HOU: Xavier Hutchinson rec O1.5 + GB@DET: Jordan Love pass TD 1+</t>
         </is>
       </c>
       <c r="B39" s="6" t="n">
-        <v>0.196</v>
+        <v>0.191</v>
       </c>
       <c r="C39" s="6" t="n">
-        <v>0.476</v>
+        <v>0.457</v>
       </c>
       <c r="D39" t="n">
-        <v>410</v>
+        <v>423</v>
       </c>
       <c r="E39" t="n">
-        <v>471</v>
+        <v>486</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>IND@MIN: Kyler Murray rush_yds U26.5 + CIN@BAL: Chase Brown rush_att O11.5 + NYG@HOU: Woody Marks rec U2.5 + GB@DET: Jared Goff pass TD 1+</t>
+          <t>IND@MIN: Kyler Murray rush_yds U26.5 + CIN@BAL: Chase Brown rush_att O11.5 + DEN@ARI: Tyler Allgeier rec U2.5 + SF@ATL: Brock Purdy pass TD 1+</t>
         </is>
       </c>
       <c r="B40" s="6" t="n">
-        <v>0.195</v>
+        <v>0.191</v>
       </c>
       <c r="C40" s="6" t="n">
-        <v>0.472</v>
+        <v>0.457</v>
       </c>
       <c r="D40" t="n">
-        <v>413</v>
+        <v>423</v>
       </c>
       <c r="E40" t="n">
-        <v>474</v>
+        <v>486</v>
       </c>
     </row>
     <row r="41"/>
@@ -1158,58 +1158,58 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>IND@MIN: Kyler Murray rush_yds U26.5 + NYG@HOU: Woody Marks rec U2.5 + SF@ATL: George Kittle anytime TD + SF@ATL: Brock Purdy pass TD 1+</t>
+          <t>IND@MIN: Kyler Murray rush_yds U26.5 + DEN@ARI: Tyler Allgeier rec U2.5 + SF@ATL: George Kittle anytime TD + SF@ATL: Brock Purdy pass TD 1+</t>
         </is>
       </c>
       <c r="B45" s="6" t="n">
-        <v>0.177</v>
+        <v>0.173</v>
       </c>
       <c r="C45" s="6" t="n">
-        <v>0.361</v>
+        <v>0.346</v>
       </c>
       <c r="D45" t="n">
-        <v>465</v>
+        <v>480</v>
       </c>
       <c r="E45" t="n">
-        <v>533</v>
+        <v>549</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CIN@BAL: Chase Brown rush_att O11.5 + NYG@HOU: Woody Marks rec U2.5 + SF@ATL: George Kittle anytime TD + SF@ATL: Brock Purdy pass TD 1+</t>
+          <t>CIN@BAL: Chase Brown rush_att O11.5 + DEN@ARI: Tyler Allgeier rec U2.5 + SF@ATL: George Kittle anytime TD + SF@ATL: Brock Purdy pass TD 1+</t>
         </is>
       </c>
       <c r="B46" s="6" t="n">
-        <v>0.177</v>
+        <v>0.173</v>
       </c>
       <c r="C46" s="6" t="n">
-        <v>0.361</v>
+        <v>0.346</v>
       </c>
       <c r="D46" t="n">
-        <v>465</v>
+        <v>480</v>
       </c>
       <c r="E46" t="n">
-        <v>533</v>
+        <v>549</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IND@MIN: Kyler Murray rush_yds U26.5 + DAL@PHI: Javonte Williams rush_att U16.5 + SF@ATL: George Kittle anytime TD + SF@ATL: Brock Purdy pass TD 1+</t>
+          <t>IND@MIN: Kyler Murray rush_yds U26.5 + NYG@HOU: Xavier Hutchinson rec O1.5 + SF@ATL: George Kittle anytime TD + SF@ATL: Brock Purdy pass TD 1+</t>
         </is>
       </c>
       <c r="B47" s="6" t="n">
-        <v>0.174</v>
+        <v>0.172</v>
       </c>
       <c r="C47" s="6" t="n">
-        <v>0.351</v>
+        <v>0.344</v>
       </c>
       <c r="D47" t="n">
-        <v>475</v>
+        <v>481</v>
       </c>
       <c r="E47" t="n">
-        <v>544</v>
+        <v>551</v>
       </c>
     </row>
     <row r="48"/>
@@ -2069,7 +2069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -2121,33 +2121,40 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>4. Availability prior. Healthy players with no designation carry p_active of about 0.95 (fitted prior), so A.J. Brown's anytime TD is 5% below his conditional number. Inactives (about 90 minutes before each kickoff) replace the prior with certainty.</t>
+          <t>3c. Log hit rates drop zero-usage games (a game with no target or carry is missing from the 'log' column), which flatters OVERs on low-volume players; red-team corrected Hooper, Dillon and Dulcich by hand. No model-versus-market gap flags: there are no prices, so no no-vig anchor exists to measure a gap against.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>5. Anytime-TD board: the 0.10 to 0.20 bin was over-predicted 2.4x in Week 6 in the sim board (frozen-run board: predicted 15.0% vs 9.1% actual, n=55) and the top ten hit 70% against 64% predicted; the W9 postmortem checks the floor. Probabilities are conditional on playing, so discount by the p_active column.</t>
+          <t>4. Availability prior. Healthy players with no designation carry p_active of about 0.95 (fitted prior), so A.J. Brown's anytime TD is 5% below his conditional number. Inactives (about 90 minutes before each kickoff) replace the prior with certainty.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>6. Minor: about two dozen practice-squad or inactive players carry small volumes at 100% active (e.g. players listed IR/PUP who appear in the unmatched-names report).</t>
+          <t>5. Anytime-TD board: the 0.10 to 0.20 bin was over-predicted 2.4x in Week 6 in the sim board (frozen-run board: predicted 15.0% vs 9.1% actual, n=55) and the top ten hit 70% against 64% predicted; the W9 postmortem checks the floor. Probabilities are conditional on playing, so discount by the p_active column.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>7. Nothing here is priced: no book prices and no touchdown prices. A PLAY is a lean at an assumed -110, not an edge. Send a screenshot of any board and I will re-price against the real numbers.</t>
+          <t>6. Minor: about two dozen practice-squad or inactive players carry small volumes at 100% active (e.g. players listed IR/PUP who appear in the unmatched-names report).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>7. Nothing here is priced: no book prices and no touchdown prices. A PLAY is a lean at an assumed -110, not an edge. Send a screenshot of any board and I will re-price against the real numbers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Method: apex-weekly run both tracks, espn_inactives.py, espn_props.py, slate_full.py sim/render, team_tables.py (box score, play-by-play and PFR advanced), league_spm.py.</t>
         </is>
@@ -13577,7 +13584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M79"/>
+  <dimension ref="A1:M52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -13606,7 +13613,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>484 lines screened: 50 PLAY (27 receiving, tagged thin: W6 receiving lines hit 35 to 52 percent, Thursday 7 of 11), 44 LEAN (the 25 best shown). Pulled by rule: receiving LEANs, pass-volume UNDERs, UNDERs on a teammate of a player now Out or Questionable ('role change'). PLAY = shrunk probability about 55.4%+ (about 61% raw), active 95%+, side cleared in at least half of the player's games. 'Agree' = the model-only track picks the same side.</t>
+          <t>484 lines screened: 23 PLAY (14 receiving, tagged thin: W6 receiving lines hit 35 to 52 percent, Thursday 7 of 11), 78 LEAN (the 25 best shown). Pulled by rule: receiving LEANs, pass-volume UNDERs, UNDERs on a teammate of a player now Out or Questionable ('role change'). PLAY = shrunk probability about 55.4%+ (about 61% raw), active 95%+, side cleared in at least half of the player's games. 'Agree' = the model-only track picks the same side.</t>
         </is>
       </c>
     </row>
@@ -13786,22 +13793,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PLAY (thin)</t>
+          <t>PLAY</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NYG@HOU</t>
+          <t>TB@CAR</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Woody Marks</t>
+          <t>Bryce Young</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>rec</t>
+          <t>rush_yds</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -13810,20 +13817,20 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.5</v>
+        <v>11.5</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.8</v>
+        <v>0.77</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>0.65</v>
+        <v>0.63</v>
       </c>
       <c r="I7" t="n">
-        <v>-184</v>
+        <v>-172</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>4/4</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -13834,29 +13841,29 @@
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>opp QB: NYG fill-in QB (J.J. McCarthy)</t>
+          <t>opp QB: TB QB1 designation (start probability 65%)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PLAY</t>
+          <t>PLAY (thin)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>DAL@PHI</t>
+          <t>DEN@ARI</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Javonte Williams</t>
+          <t>Tyler Allgeier</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>rush_att</t>
+          <t>rec</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -13865,20 +13872,20 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>16.5</v>
+        <v>2.5</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.77</v>
+        <v>0.76</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>0.64</v>
+        <v>0.63</v>
       </c>
       <c r="I8" t="n">
-        <v>-175</v>
+        <v>-171</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -13887,31 +13894,27 @@
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>opp QB: PHI fill-in QB (Tanner McKee)</t>
-        </is>
-      </c>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PLAY</t>
+          <t>PLAY (thin)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DEN@ARI</t>
+          <t>NYG@HOU</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Jacoby Brissett</t>
+          <t>Xavier Hutchinson</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>rush_yds</t>
+          <t>rec</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -13920,20 +13923,20 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>6.5</v>
+        <v>1.5</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.77</v>
+        <v>0.76</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>0.63</v>
       </c>
       <c r="I9" t="n">
-        <v>-173</v>
+        <v>-170</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -13942,7 +13945,11 @@
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>opp QB: NYG fill-in QB (J.J. McCarthy)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -13952,12 +13959,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>TB@CAR</t>
+          <t>GB@DET</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Bryce Young</t>
+          <t>Jordan Love</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -13971,20 +13978,20 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>11.5</v>
+        <v>6.5</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.77</v>
+        <v>0.75</v>
       </c>
       <c r="H10" s="6" t="n">
         <v>0.63</v>
       </c>
       <c r="I10" t="n">
-        <v>-172</v>
+        <v>-168</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>4/4</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -13993,11 +14000,7 @@
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>opp QB: TB QB1 designation (start probability 65%)</t>
-        </is>
-      </c>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -14007,39 +14010,39 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>DEN@ARI</t>
+          <t>NYG@HOU</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tyler Allgeier</t>
+          <t>Kayshon Boutte</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>rec</t>
+          <t>rec_yds</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>UNDER</t>
+          <t>OVER</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.5</v>
+        <v>9.5</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="H11" s="6" t="n">
         <v>0.63</v>
       </c>
       <c r="I11" t="n">
-        <v>-171</v>
+        <v>-167</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -14048,7 +14051,11 @@
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>opp QB: NYG fill-in QB (J.J. McCarthy)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -14058,12 +14065,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>NYG@HOU</t>
+          <t>LA@LV</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Xavier Hutchinson</t>
+          <t>Kyren Williams</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -14077,20 +14084,20 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>0.76</v>
+        <v>0.73</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>0.63</v>
+        <v>0.62</v>
       </c>
       <c r="I12" t="n">
-        <v>-170</v>
+        <v>-161</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -14099,11 +14106,7 @@
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>opp QB: NYG fill-in QB (J.J. McCarthy)</t>
-        </is>
-      </c>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -14113,17 +14116,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>GB@DET</t>
+          <t>LA@LV</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Jordan Love</t>
+          <t>Kyren Williams</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>rush_yds</t>
+          <t>rush_att</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -14132,20 +14135,20 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>6.5</v>
+        <v>15.5</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>0.75</v>
+        <v>0.72</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>0.63</v>
+        <v>0.61</v>
       </c>
       <c r="I13" t="n">
-        <v>-168</v>
+        <v>-157</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -14159,44 +14162,44 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PLAY</t>
+          <t>PLAY (thin)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>KC@SEA</t>
+          <t>GB@DET</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>George Holani</t>
+          <t>Amon-Ra St. Brown</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>rush_yds</t>
+          <t>rec_yds</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>OVER</t>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>13.5</v>
+        <v>84.5</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>0.75</v>
+        <v>0.72</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>0.63</v>
+        <v>0.61</v>
       </c>
       <c r="I14" t="n">
-        <v>-168</v>
+        <v>-157</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -14210,22 +14213,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PLAY</t>
+          <t>PLAY (thin)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CLE@TEN</t>
+          <t>CIN@BAL</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Quinshon Judkins</t>
+          <t>Ja'Marr Chase</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>rush_att</t>
+          <t>rec</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -14234,20 +14237,20 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>14.5</v>
+        <v>7.5</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>0.75</v>
+        <v>0.72</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>0.63</v>
+        <v>0.61</v>
       </c>
       <c r="I15" t="n">
-        <v>-168</v>
+        <v>-156</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -14256,7 +14259,11 @@
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>opp QB: BAL fill-in QB (QB1 Out)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -14266,17 +14273,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>NYG@HOU</t>
+          <t>KC@SEA</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Kayshon Boutte</t>
+          <t>Noah Gray</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>rec_yds</t>
+          <t>rec</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -14285,20 +14292,20 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>9.5</v>
+        <v>1.5</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>0.75</v>
+        <v>0.7</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>0.63</v>
+        <v>0.6</v>
       </c>
       <c r="I16" t="n">
-        <v>-167</v>
+        <v>-150</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -14307,31 +14314,27 @@
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>opp QB: NYG fill-in QB (J.J. McCarthy)</t>
-        </is>
-      </c>
+      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PLAY</t>
+          <t>PLAY (thin)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CIN@BAL</t>
+          <t>TB@CAR</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Samaje Perine</t>
+          <t>Chuba Hubbard</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>rush_att</t>
+          <t>rec</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -14340,20 +14343,20 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>7.5</v>
+        <v>2.5</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>0.74</v>
+        <v>0.7</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>0.62</v>
+        <v>0.6</v>
       </c>
       <c r="I17" t="n">
-        <v>-162</v>
+        <v>-150</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -14364,29 +14367,29 @@
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
-          <t>opp QB: BAL fill-in QB (QB1 Out)</t>
+          <t>opp QB: TB QB1 designation (start probability 65%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PLAY (thin)</t>
+          <t>PLAY</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>LA@LV</t>
+          <t>PIT@NO</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Kyren Williams</t>
+          <t>Alvin Kamara</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>rec</t>
+          <t>rush_yds</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -14395,20 +14398,20 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>3.5</v>
+        <v>17.5</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>0.73</v>
+        <v>0.68</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>0.62</v>
+        <v>0.59</v>
       </c>
       <c r="I18" t="n">
-        <v>-161</v>
+        <v>-145</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -14427,12 +14430,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>TB@CAR</t>
+          <t>NYG@HOU</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Tommy Tremble</t>
+          <t>Marvin Harrison Jr.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -14442,24 +14445,24 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>OVER</t>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="G19" s="6" t="n">
-        <v>0.73</v>
+        <v>0.67</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>0.61</v>
+        <v>0.58</v>
       </c>
       <c r="I19" t="n">
-        <v>-160</v>
+        <v>-141</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -14470,7 +14473,7 @@
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
-          <t>opp QB: TB QB1 designation (start probability 65%)</t>
+          <t>opp QB: NYG fill-in QB (J.J. McCarthy)</t>
         </is>
       </c>
     </row>
@@ -14482,12 +14485,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PIT@NO</t>
+          <t>DEN@ARI</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Germie Bernard</t>
+          <t>Courtland Sutton</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -14501,20 +14504,20 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>5.5</v>
+        <v>3.5</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>0.73</v>
+        <v>0.66</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>0.61</v>
+        <v>0.58</v>
       </c>
       <c r="I20" t="n">
-        <v>-159</v>
+        <v>-138</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -14533,39 +14536,39 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>LA@LV</t>
+          <t>PIT@NO</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Kyren Williams</t>
+          <t>Aaron Rodgers</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>rush_att</t>
+          <t>pass_cmp</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>UNDER</t>
+          <t>OVER</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>15.5</v>
+        <v>21.5</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>0.72</v>
+        <v>0.65</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>0.61</v>
+        <v>0.58</v>
       </c>
       <c r="I21" t="n">
-        <v>-157</v>
+        <v>-136</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -14589,7 +14592,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Amon-Ra St. Brown</t>
+          <t>Jameson Williams</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -14603,16 +14606,16 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>84.5</v>
+        <v>54.5</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>0.72</v>
+        <v>0.65</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>0.61</v>
+        <v>0.57</v>
       </c>
       <c r="I22" t="n">
-        <v>-157</v>
+        <v>-134</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -14630,40 +14633,40 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PLAY (thin)</t>
+          <t>PLAY</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CIN@BAL</t>
+          <t>KC@SEA</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Ja'Marr Chase</t>
+          <t>Kenneth Walker III</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>rec</t>
+          <t>rush_yds</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>UNDER</t>
+          <t>OVER</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>7.5</v>
+        <v>80.5</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>0.72</v>
+        <v>0.64</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>0.61</v>
+        <v>0.57</v>
       </c>
       <c r="I23" t="n">
-        <v>-156</v>
+        <v>-132</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -14676,31 +14679,27 @@
         </is>
       </c>
       <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>opp QB: BAL fill-in QB (QB1 Out)</t>
-        </is>
-      </c>
+      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>PLAY</t>
+          <t>PLAY (thin)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>KC@SEA</t>
+          <t>TB@CAR</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Emmett Johnson</t>
+          <t>John Metchie III</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>rush_yds</t>
+          <t>rec_yds</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -14709,20 +14708,20 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>0.71</v>
+        <v>0.64</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>0.61</v>
+        <v>0.57</v>
       </c>
       <c r="I24" t="n">
-        <v>-154</v>
+        <v>-131</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>3/4</t>
+          <t>3/3</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -14731,27 +14730,31 @@
         </is>
       </c>
       <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>opp QB: TB QB1 designation (start probability 65%)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>PLAY</t>
+          <t>PLAY (thin)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>NYG@HOU</t>
+          <t>DEN@ARI</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>C.J. Stroud</t>
+          <t>Trey McBride</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>rush_yds</t>
+          <t>rec</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -14760,20 +14763,20 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>9.5</v>
+        <v>6.5</v>
       </c>
       <c r="G25" s="6" t="n">
-        <v>0.7</v>
+        <v>0.64</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>0.6</v>
+        <v>0.57</v>
       </c>
       <c r="I25" t="n">
-        <v>-151</v>
+        <v>-131</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -14782,31 +14785,27 @@
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>opp QB: NYG fill-in QB (J.J. McCarthy)</t>
-        </is>
-      </c>
+      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PLAY (thin)</t>
+          <t>PLAY</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>NYG@HOU</t>
+          <t>DEN@ARI</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Jaylin Noel</t>
+          <t>Bo Nix</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>rec</t>
+          <t>rush_yds</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -14815,20 +14814,20 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>2.5</v>
+        <v>10.5</v>
       </c>
       <c r="G26" s="6" t="n">
-        <v>0.7</v>
+        <v>0.63</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>0.6</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I26" t="n">
-        <v>-151</v>
+        <v>-130</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -14837,11 +14836,7 @@
         </is>
       </c>
       <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>opp QB: NYG fill-in QB (J.J. McCarthy)</t>
-        </is>
-      </c>
+      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -14851,12 +14846,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>KC@SEA</t>
+          <t>IND@MIN</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Noah Gray</t>
+          <t>Jauan Jennings</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -14866,24 +14861,24 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>OVER</t>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="F27" t="n">
         <v>1.5</v>
       </c>
       <c r="G27" s="6" t="n">
-        <v>0.7</v>
+        <v>0.61</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>0.6</v>
+        <v>0.55</v>
       </c>
       <c r="I27" t="n">
-        <v>-150</v>
+        <v>-125</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>4/4</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -14897,22 +14892,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>PLAY (thin)</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>TB@CAR</t>
+          <t>DAL@PHI</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Chuba Hubbard</t>
+          <t>Saquon Barkley</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>rec</t>
+          <t>rush_yds</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -14921,20 +14916,20 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.5</v>
+        <v>70.5</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>0.7</v>
+        <v>0.92</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>0.6</v>
+        <v>0.71</v>
       </c>
       <c r="I28" t="n">
-        <v>-150</v>
+        <v>-244</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>2/4</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -14942,32 +14937,36 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>same bet as sibling line</t>
+        </is>
+      </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>opp QB: TB QB1 designation (start probability 65%)</t>
+          <t>fill-in QB (Tanner McKee)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>PLAY (thin)</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>TB@CAR</t>
+          <t>CLE@TEN</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Jalen Coker</t>
+          <t>Deshaun Watson</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>rec_yds</t>
+          <t>rush_yds</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -14976,20 +14975,20 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>69.5</v>
+        <v>29.5</v>
       </c>
       <c r="G29" s="6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.85</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>0.59</v>
+        <v>0.67</v>
       </c>
       <c r="I29" t="n">
-        <v>-147</v>
+        <v>-207</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2/4</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -14997,17 +14996,17 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>opp QB: TB QB1 designation (start probability 65%)</t>
-        </is>
-      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>same bet as sibling line</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PLAY (thin)</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -15017,34 +15016,34 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Jake Ferguson</t>
+          <t>Javonte Williams</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>rec_yds</t>
+          <t>rush_att</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>OVER</t>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>18.5</v>
+        <v>16.5</v>
       </c>
       <c r="G30" s="6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.77</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>0.59</v>
+        <v>0.64</v>
       </c>
       <c r="I30" t="n">
-        <v>-146</v>
+        <v>-175</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -15052,7 +15051,11 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>same bet as sibling line</t>
+        </is>
+      </c>
       <c r="M30" t="inlineStr">
         <is>
           <t>opp QB: PHI fill-in QB (Tanner McKee)</t>
@@ -15062,44 +15065,44 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PLAY</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PIT@NO</t>
+          <t>CIN@BAL</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Alvin Kamara</t>
+          <t>Tyler Huntley</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>rush_yds</t>
+          <t>rush_att</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>OVER</t>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>17.5</v>
+        <v>5.5</v>
       </c>
       <c r="G31" s="6" t="n">
-        <v>0.68</v>
+        <v>0.77</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>0.59</v>
+        <v>0.64</v>
       </c>
       <c r="I31" t="n">
-        <v>-145</v>
+        <v>-174</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>2/3</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -15108,22 +15111,26 @@
         </is>
       </c>
       <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>fill-in QB (QB1 Out)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>PLAY</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>GB@DET</t>
+          <t>DEN@ARI</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Sione Vaki</t>
+          <t>Jacoby Brissett</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -15137,20 +15144,20 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>8.5</v>
+        <v>6.5</v>
       </c>
       <c r="G32" s="6" t="n">
-        <v>0.68</v>
+        <v>0.77</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>0.59</v>
+        <v>0.63</v>
       </c>
       <c r="I32" t="n">
-        <v>-145</v>
+        <v>-173</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2/4</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -15158,13 +15165,17 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>red-team downgrade</t>
+        </is>
+      </c>
       <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>PLAY</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -15174,7 +15185,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Tony Pollard</t>
+          <t>Quinshon Judkins</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -15188,20 +15199,20 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>17.5</v>
+        <v>14.5</v>
       </c>
       <c r="G33" s="6" t="n">
-        <v>0.68</v>
+        <v>0.75</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>0.59</v>
+        <v>0.63</v>
       </c>
       <c r="I33" t="n">
-        <v>-145</v>
+        <v>-168</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -15209,50 +15220,54 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr"/>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>same bet as sibling line</t>
+        </is>
+      </c>
       <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>PLAY (thin)</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>NYG@HOU</t>
+          <t>CIN@BAL</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Marvin Harrison Jr.</t>
+          <t>Tyler Huntley</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>rec</t>
+          <t>pass_yds</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>UNDER</t>
+          <t>OVER</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>2.5</v>
+        <v>197.5</v>
       </c>
       <c r="G34" s="6" t="n">
-        <v>0.67</v>
+        <v>0.73</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>0.58</v>
+        <v>0.62</v>
       </c>
       <c r="I34" t="n">
-        <v>-141</v>
+        <v>-160</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>1/3</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -15263,29 +15278,29 @@
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr">
         <is>
-          <t>opp QB: NYG fill-in QB (J.J. McCarthy)</t>
+          <t>fill-in QB (QB1 Out)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>PLAY (thin)</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PIT@NO</t>
+          <t>SF@ATL</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Devaughn Vele</t>
+          <t>Michael Penix Jr.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>rec_yds</t>
+          <t>pass_att</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -15294,20 +15309,20 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>42.5</v>
+        <v>31.5</v>
       </c>
       <c r="G35" s="6" t="n">
-        <v>0.67</v>
+        <v>0.72</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>0.58</v>
+        <v>0.61</v>
       </c>
       <c r="I35" t="n">
-        <v>-140</v>
+        <v>-156</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>2/4</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -15315,28 +15330,32 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>same bet as sibling line</t>
+        </is>
+      </c>
       <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PLAY (thin)</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>DEN@ARI</t>
+          <t>DAL@PHI</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Courtland Sutton</t>
+          <t>Javonte Williams</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>rec</t>
+          <t>rush_yds</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -15345,20 +15364,20 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>3.5</v>
+        <v>65.5</v>
       </c>
       <c r="G36" s="6" t="n">
-        <v>0.66</v>
+        <v>0.71</v>
       </c>
       <c r="H36" s="6" t="n">
-        <v>0.58</v>
+        <v>0.61</v>
       </c>
       <c r="I36" t="n">
-        <v>-138</v>
+        <v>-154</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -15366,28 +15385,36 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>same bet as sibling line</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>opp QB: PHI fill-in QB (Tanner McKee)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>PLAY</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PIT@NO</t>
+          <t>KC@SEA</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Aaron Rodgers</t>
+          <t>Emmett Johnson</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>pass_cmp</t>
+          <t>rush_yds</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -15396,20 +15423,20 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>21.5</v>
+        <v>8.5</v>
       </c>
       <c r="G37" s="6" t="n">
-        <v>0.65</v>
+        <v>0.71</v>
       </c>
       <c r="H37" s="6" t="n">
-        <v>0.58</v>
+        <v>0.61</v>
       </c>
       <c r="I37" t="n">
-        <v>-136</v>
+        <v>-154</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>5/6</t>
+          <t>3/4</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -15417,28 +15444,32 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr"/>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>red-team downgrade</t>
+        </is>
+      </c>
       <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>PLAY</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>LA@LV</t>
+          <t>DAL@PHI</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Blake Corum</t>
+          <t>Dak Prescott</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>rush_att</t>
+          <t>rush_yds</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -15447,20 +15478,20 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>8.5</v>
+        <v>9.5</v>
       </c>
       <c r="G38" s="6" t="n">
-        <v>0.65</v>
+        <v>0.71</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>0.58</v>
+        <v>0.6</v>
       </c>
       <c r="I38" t="n">
-        <v>-136</v>
+        <v>-153</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -15468,28 +15499,36 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>same bet as sibling line</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>opp QB: PHI fill-in QB (Tanner McKee)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>PLAY (thin)</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>GB@DET</t>
+          <t>SF@ATL</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Jameson Williams</t>
+          <t>Brock Purdy</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>rec_yds</t>
+          <t>rush_att</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -15498,20 +15537,20 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>54.5</v>
+        <v>4.5</v>
       </c>
       <c r="G39" s="6" t="n">
-        <v>0.65</v>
+        <v>0.71</v>
       </c>
       <c r="H39" s="6" t="n">
-        <v>0.57</v>
+        <v>0.6</v>
       </c>
       <c r="I39" t="n">
-        <v>-134</v>
+        <v>-152</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>2/6</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -15519,50 +15558,54 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr"/>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>same bet as sibling line</t>
+        </is>
+      </c>
       <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>PLAY (thin)</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>DAL@PHI</t>
+          <t>NYG@HOU</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>CeeDee Lamb</t>
+          <t>C.J. Stroud</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>rec</t>
+          <t>rush_yds</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>UNDER</t>
+          <t>OVER</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>7.5</v>
+        <v>9.5</v>
       </c>
       <c r="G40" s="6" t="n">
-        <v>0.64</v>
+        <v>0.7</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>0.57</v>
+        <v>0.6</v>
       </c>
       <c r="I40" t="n">
-        <v>-133</v>
+        <v>-151</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -15570,54 +15613,58 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="L40" t="inlineStr"/>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>red-team downgrade</t>
+        </is>
+      </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>opp QB: PHI fill-in QB (Tanner McKee)</t>
+          <t>opp QB: NYG fill-in QB (J.J. McCarthy)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>PLAY</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>KC@SEA</t>
+          <t>TB@CAR</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Kenneth Walker III</t>
+          <t>Chuba Hubbard</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>rush_yds</t>
+          <t>rush_att</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>OVER</t>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>80.5</v>
+        <v>17.5</v>
       </c>
       <c r="G41" s="6" t="n">
-        <v>0.64</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H41" s="6" t="n">
-        <v>0.57</v>
+        <v>0.59</v>
       </c>
       <c r="I41" t="n">
-        <v>-132</v>
+        <v>-146</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -15626,49 +15673,53 @@
         </is>
       </c>
       <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>opp QB: TB QB1 designation (start probability 65%)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>PLAY (thin)</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>MIA@NYJ</t>
+          <t>GB@DET</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Garrett Wilson</t>
+          <t>Sione Vaki</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>rec_yds</t>
+          <t>rush_yds</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>UNDER</t>
+          <t>OVER</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>64.5</v>
+        <v>8.5</v>
       </c>
       <c r="G42" s="6" t="n">
-        <v>0.64</v>
+        <v>0.68</v>
       </c>
       <c r="H42" s="6" t="n">
-        <v>0.57</v>
+        <v>0.59</v>
       </c>
       <c r="I42" t="n">
-        <v>-132</v>
+        <v>-145</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>3/6</t>
+          <t>2/4</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -15676,28 +15727,32 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr"/>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>red-team downgrade</t>
+        </is>
+      </c>
       <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>PLAY</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>TB@CAR</t>
+          <t>DAL@PHI</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>AJ Dillon</t>
+          <t>Tanner McKee</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>rush_att</t>
+          <t>pass_cmp</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -15706,20 +15761,20 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.5</v>
+        <v>19.5</v>
       </c>
       <c r="G43" s="6" t="n">
-        <v>0.64</v>
+        <v>0.68</v>
       </c>
       <c r="H43" s="6" t="n">
-        <v>0.57</v>
+        <v>0.59</v>
       </c>
       <c r="I43" t="n">
-        <v>-131</v>
+        <v>-145</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>3/4</t>
+          <t>1/1</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -15727,32 +15782,36 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr"/>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>same bet as sibling line</t>
+        </is>
+      </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>opp QB: TB QB1 designation (start probability 65%)</t>
+          <t>fill-in QB (Tanner McKee)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PLAY (thin)</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>TB@CAR</t>
+          <t>CIN@BAL</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>John Metchie III</t>
+          <t>Chase Brown</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>rec_yds</t>
+          <t>rush_yds</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -15761,20 +15820,20 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>10.5</v>
+        <v>41.5</v>
       </c>
       <c r="G44" s="6" t="n">
-        <v>0.64</v>
+        <v>0.68</v>
       </c>
       <c r="H44" s="6" t="n">
-        <v>0.57</v>
+        <v>0.59</v>
       </c>
       <c r="I44" t="n">
-        <v>-131</v>
+        <v>-145</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>3/3</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -15782,54 +15841,58 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr"/>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>same bet as sibling line</t>
+        </is>
+      </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>opp QB: TB QB1 designation (start probability 65%)</t>
+          <t>opp QB: BAL fill-in QB (QB1 Out)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>PLAY (thin)</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>DEN@ARI</t>
+          <t>CLE@TEN</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Trey McBride</t>
+          <t>Tony Pollard</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>rec</t>
+          <t>rush_att</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>OVER</t>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>6.5</v>
+        <v>17.5</v>
       </c>
       <c r="G45" s="6" t="n">
-        <v>0.64</v>
+        <v>0.68</v>
       </c>
       <c r="H45" s="6" t="n">
-        <v>0.57</v>
+        <v>0.59</v>
       </c>
       <c r="I45" t="n">
-        <v>-131</v>
+        <v>-145</v>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -15837,50 +15900,54 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr"/>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>red-team downgrade</t>
+        </is>
+      </c>
       <c r="M45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>PLAY</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>LA@LV</t>
+          <t>CLE@TEN</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Ashton Jeanty</t>
+          <t>Quinshon Judkins</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>rush_att</t>
+          <t>rush_yds</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>OVER</t>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>14.5</v>
+        <v>46.5</v>
       </c>
       <c r="G46" s="6" t="n">
-        <v>0.63</v>
+        <v>0.67</v>
       </c>
       <c r="H46" s="6" t="n">
-        <v>0.57</v>
+        <v>0.59</v>
       </c>
       <c r="I46" t="n">
-        <v>-130</v>
+        <v>-142</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>4/6</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -15888,50 +15955,54 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr"/>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>same bet as sibling line</t>
+        </is>
+      </c>
       <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>PLAY</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>DEN@ARI</t>
+          <t>NYG@HOU</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Bo Nix</t>
+          <t>Woody Marks</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>rush_yds</t>
+          <t>rush_att</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>UNDER</t>
+          <t>OVER</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>10.5</v>
+        <v>16.5</v>
       </c>
       <c r="G47" s="6" t="n">
-        <v>0.63</v>
+        <v>0.67</v>
       </c>
       <c r="H47" s="6" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.59</v>
       </c>
       <c r="I47" t="n">
-        <v>-130</v>
+        <v>-141</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>6/6</t>
+          <t>0/6</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -15940,49 +16011,53 @@
         </is>
       </c>
       <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>opp QB: NYG fill-in QB (J.J. McCarthy)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>PLAY</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>MIA@NYJ</t>
+          <t>DAL@PHI</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Malik Willis</t>
+          <t>Tanner McKee</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>rush_att</t>
+          <t>pass_yds</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>UNDER</t>
+          <t>OVER</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>6.5</v>
+        <v>192.5</v>
       </c>
       <c r="G48" s="6" t="n">
-        <v>0.63</v>
+        <v>0.67</v>
       </c>
       <c r="H48" s="6" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.58</v>
       </c>
       <c r="I48" t="n">
-        <v>-129</v>
+        <v>-140</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>1/1</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -15990,23 +16065,31 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>same bet as sibling line</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>fill-in QB (Tanner McKee)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>PLAY</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>DEN@ARI</t>
+          <t>NYG@HOU</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>RJ Harvey</t>
+          <t>Woody Marks</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -16020,20 +16103,20 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>14.5</v>
+        <v>63.5</v>
       </c>
       <c r="G49" s="6" t="n">
-        <v>0.63</v>
+        <v>0.65</v>
       </c>
       <c r="H49" s="6" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.58</v>
       </c>
       <c r="I49" t="n">
-        <v>-129</v>
+        <v>-136</v>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>0/6</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -16042,27 +16125,31 @@
         </is>
       </c>
       <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>opp QB: NYG fill-in QB (J.J. McCarthy)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>PLAY (thin)</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>CIN@BAL</t>
+          <t>CLE@TEN</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Dohnte Meyers</t>
+          <t>Tyjae Spears</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>rec_yds</t>
+          <t>rush_yds</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -16071,20 +16158,20 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>13.5</v>
+        <v>9.5</v>
       </c>
       <c r="G50" s="6" t="n">
-        <v>0.62</v>
+        <v>0.65</v>
       </c>
       <c r="H50" s="6" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.58</v>
       </c>
       <c r="I50" t="n">
-        <v>-128</v>
+        <v>-136</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>2/6</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -16092,50 +16179,50 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>opp QB: BAL fill-in QB (QB1 Out)</t>
-        </is>
-      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>same bet as sibling line</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>PLAY (thin)</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CLE@TEN</t>
+          <t>LA@LV</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Elic Ayomanor</t>
+          <t>Blake Corum</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>rec_yds</t>
+          <t>rush_att</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>OVER</t>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>16.5</v>
+        <v>8.5</v>
       </c>
       <c r="G51" s="6" t="n">
-        <v>0.61</v>
+        <v>0.65</v>
       </c>
       <c r="H51" s="6" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.58</v>
       </c>
       <c r="I51" t="n">
-        <v>-125</v>
+        <v>-136</v>
       </c>
       <c r="J51" t="inlineStr">
         <is>
@@ -16147,13 +16234,17 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="L51" t="inlineStr"/>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>red-team downgrade</t>
+        </is>
+      </c>
       <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>PLAY (thin)</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -16163,34 +16254,34 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Austin Hooper</t>
+          <t>Brock Purdy</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>rec</t>
+          <t>rush_yds</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>OVER</t>
+          <t>UNDER</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>0.5</v>
+        <v>19.5</v>
       </c>
       <c r="G52" s="6" t="n">
-        <v>0.61</v>
+        <v>0.65</v>
       </c>
       <c r="H52" s="6" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.58</v>
       </c>
       <c r="I52" t="n">
-        <v>-125</v>
+        <v>-135</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>4/4</t>
+          <t>1/6</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -16198,1453 +16289,12 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="L52" t="inlineStr"/>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>same bet as sibling line</t>
+        </is>
+      </c>
       <c r="M52" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>PLAY (thin)</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>MIA@NYJ</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Greg Dulcich</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>rec_yds</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>OVER</t>
-        </is>
-      </c>
-      <c r="F53" t="n">
-        <v>21.5</v>
-      </c>
-      <c r="G53" s="6" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="H53" s="6" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="I53" t="n">
-        <v>-125</v>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>2/4</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>PLAY (thin)</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>IND@MIN</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Jauan Jennings</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>rec</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>UNDER</t>
-        </is>
-      </c>
-      <c r="F54" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G54" s="6" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="H54" s="6" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="I54" t="n">
-        <v>-125</v>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>4/4</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>CLE@TEN</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Deshaun Watson</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>rush_yds</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>UNDER</t>
-        </is>
-      </c>
-      <c r="F55" t="n">
-        <v>29.5</v>
-      </c>
-      <c r="G55" s="6" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="H55" s="6" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="I55" t="n">
-        <v>-207</v>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>3/6</t>
-        </is>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>model vs own record</t>
-        </is>
-      </c>
-      <c r="M55" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>CIN@BAL</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Tyler Huntley</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>rush_att</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>UNDER</t>
-        </is>
-      </c>
-      <c r="F56" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="G56" s="6" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="H56" s="6" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="I56" t="n">
-        <v>-174</v>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>2/3</t>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr">
-        <is>
-          <t>fill-in QB (QB1 Out)</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>CIN@BAL</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Tyler Huntley</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>pass_yds</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>OVER</t>
-        </is>
-      </c>
-      <c r="F57" t="n">
-        <v>197.5</v>
-      </c>
-      <c r="G57" s="6" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="H57" s="6" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="I57" t="n">
-        <v>-160</v>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>1/3</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr">
-        <is>
-          <t>fill-in QB (QB1 Out)</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>DAL@PHI</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Javonte Williams</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>rush_yds</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>UNDER</t>
-        </is>
-      </c>
-      <c r="F58" t="n">
-        <v>65.5</v>
-      </c>
-      <c r="G58" s="6" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="H58" s="6" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="I58" t="n">
-        <v>-154</v>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>5/6</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L58" t="inlineStr">
-        <is>
-          <t>same bet as sibling line</t>
-        </is>
-      </c>
-      <c r="M58" t="inlineStr">
-        <is>
-          <t>opp QB: PHI fill-in QB (Tanner McKee)</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>DAL@PHI</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Dak Prescott</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>rush_yds</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>UNDER</t>
-        </is>
-      </c>
-      <c r="F59" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="G59" s="6" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="H59" s="6" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="I59" t="n">
-        <v>-153</v>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>2/5</t>
-        </is>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr">
-        <is>
-          <t>opp QB: PHI fill-in QB (Tanner McKee)</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>SF@ATL</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Brock Purdy</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>rush_att</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>UNDER</t>
-        </is>
-      </c>
-      <c r="F60" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="G60" s="6" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="H60" s="6" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="I60" t="n">
-        <v>-152</v>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>2/6</t>
-        </is>
-      </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>TB@CAR</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Chuba Hubbard</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>rush_att</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>UNDER</t>
-        </is>
-      </c>
-      <c r="F61" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="G61" s="6" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="H61" s="6" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="I61" t="n">
-        <v>-146</v>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>2/5</t>
-        </is>
-      </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L61" t="inlineStr"/>
-      <c r="M61" t="inlineStr">
-        <is>
-          <t>opp QB: TB QB1 designation (start probability 65%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>CIN@BAL</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Chase Brown</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>rush_yds</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>OVER</t>
-        </is>
-      </c>
-      <c r="F62" t="n">
-        <v>41.5</v>
-      </c>
-      <c r="G62" s="6" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="H62" s="6" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="I62" t="n">
-        <v>-145</v>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>3/5</t>
-        </is>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>same bet as sibling line</t>
-        </is>
-      </c>
-      <c r="M62" t="inlineStr">
-        <is>
-          <t>opp QB: BAL fill-in QB (QB1 Out)</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>CLE@TEN</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Quinshon Judkins</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>rush_yds</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>UNDER</t>
-        </is>
-      </c>
-      <c r="F63" t="n">
-        <v>46.5</v>
-      </c>
-      <c r="G63" s="6" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="H63" s="6" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="I63" t="n">
-        <v>-142</v>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>3/5</t>
-        </is>
-      </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t>same bet as sibling line</t>
-        </is>
-      </c>
-      <c r="M63" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>NYG@HOU</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Woody Marks</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>rush_att</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>OVER</t>
-        </is>
-      </c>
-      <c r="F64" t="n">
-        <v>16.5</v>
-      </c>
-      <c r="G64" s="6" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="H64" s="6" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="I64" t="n">
-        <v>-141</v>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>0/6</t>
-        </is>
-      </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L64" t="inlineStr"/>
-      <c r="M64" t="inlineStr">
-        <is>
-          <t>opp QB: NYG fill-in QB (J.J. McCarthy)</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>NYG@HOU</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Woody Marks</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>rush_yds</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>OVER</t>
-        </is>
-      </c>
-      <c r="F65" t="n">
-        <v>63.5</v>
-      </c>
-      <c r="G65" s="6" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="H65" s="6" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="I65" t="n">
-        <v>-136</v>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>0/6</t>
-        </is>
-      </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="inlineStr">
-        <is>
-          <t>opp QB: NYG fill-in QB (J.J. McCarthy)</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>SF@ATL</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Brock Purdy</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>rush_yds</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>UNDER</t>
-        </is>
-      </c>
-      <c r="F66" t="n">
-        <v>19.5</v>
-      </c>
-      <c r="G66" s="6" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="H66" s="6" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="I66" t="n">
-        <v>-135</v>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>1/6</t>
-        </is>
-      </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>PIT@NO</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>Tyler Shough</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>rush_att</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>UNDER</t>
-        </is>
-      </c>
-      <c r="F67" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="G67" s="6" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="H67" s="6" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="I67" t="n">
-        <v>-133</v>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>2/5</t>
-        </is>
-      </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>PIT@NO</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>Tyler Shough</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>rush_yds</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>UNDER</t>
-        </is>
-      </c>
-      <c r="F68" t="n">
-        <v>14.5</v>
-      </c>
-      <c r="G68" s="6" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="H68" s="6" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="I68" t="n">
-        <v>-131</v>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>2/5</t>
-        </is>
-      </c>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>MIA@NYJ</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>Malik Willis</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>pass_att</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>OVER</t>
-        </is>
-      </c>
-      <c r="F69" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="G69" s="6" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="H69" s="6" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="I69" t="n">
-        <v>-128</v>
-      </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>1/5</t>
-        </is>
-      </c>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L69" t="inlineStr"/>
-      <c r="M69" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>MIA@NYJ</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>Geno Smith</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>pass_cmp</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>OVER</t>
-        </is>
-      </c>
-      <c r="F70" t="n">
-        <v>20.5</v>
-      </c>
-      <c r="G70" s="6" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="H70" s="6" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="I70" t="n">
-        <v>-128</v>
-      </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>2/6</t>
-        </is>
-      </c>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L70" t="inlineStr"/>
-      <c r="M70" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>TB@CAR</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>Bucky Irving</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>rush_yds</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>OVER</t>
-        </is>
-      </c>
-      <c r="F71" t="n">
-        <v>65.5</v>
-      </c>
-      <c r="G71" s="6" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="H71" s="6" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="I71" t="n">
-        <v>-126</v>
-      </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>2/6</t>
-        </is>
-      </c>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L71" t="inlineStr"/>
-      <c r="M71" t="inlineStr">
-        <is>
-          <t>QB1 designation (start probability 65%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>TB@CAR</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>Sean Tucker</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>rush_yds</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>UNDER</t>
-        </is>
-      </c>
-      <c r="F72" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="G72" s="6" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="H72" s="6" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="I72" t="n">
-        <v>-125</v>
-      </c>
-      <c r="J72" t="inlineStr">
-        <is>
-          <t>0/2</t>
-        </is>
-      </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L72" t="inlineStr"/>
-      <c r="M72" t="inlineStr">
-        <is>
-          <t>QB1 designation (start probability 65%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>CIN@BAL</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>Tyler Huntley</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>pass_att</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>OVER</t>
-        </is>
-      </c>
-      <c r="F73" t="n">
-        <v>28.5</v>
-      </c>
-      <c r="G73" s="6" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="H73" s="6" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="I73" t="n">
-        <v>-125</v>
-      </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>2/3</t>
-        </is>
-      </c>
-      <c r="K73" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="L73" t="inlineStr"/>
-      <c r="M73" t="inlineStr">
-        <is>
-          <t>fill-in QB (QB1 Out)</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>GB@DET</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>Jahmyr Gibbs</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>rush_yds</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>UNDER</t>
-        </is>
-      </c>
-      <c r="F74" t="n">
-        <v>97.5</v>
-      </c>
-      <c r="G74" s="6" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="H74" s="6" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="I74" t="n">
-        <v>-125</v>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>2/5</t>
-        </is>
-      </c>
-      <c r="K74" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L74" t="inlineStr"/>
-      <c r="M74" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>DAL@PHI</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>Dak Prescott</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>pass_cmp</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>OVER</t>
-        </is>
-      </c>
-      <c r="F75" t="n">
-        <v>23.5</v>
-      </c>
-      <c r="G75" s="6" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="H75" s="6" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="I75" t="n">
-        <v>-123</v>
-      </c>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>5/6</t>
-        </is>
-      </c>
-      <c r="K75" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L75" t="inlineStr"/>
-      <c r="M75" t="inlineStr">
-        <is>
-          <t>opp QB: PHI fill-in QB (Tanner McKee)</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>PIT@NO</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>Kendre Miller</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>rush_att</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>UNDER</t>
-        </is>
-      </c>
-      <c r="F76" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="G76" s="6" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H76" s="6" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="I76" t="n">
-        <v>-123</v>
-      </c>
-      <c r="J76" t="inlineStr">
-        <is>
-          <t>4/5</t>
-        </is>
-      </c>
-      <c r="K76" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L76" t="inlineStr"/>
-      <c r="M76" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>MIA@NYJ</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>Jaylen Wright</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>rush_yds</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>OVER</t>
-        </is>
-      </c>
-      <c r="F77" t="n">
-        <v>15.5</v>
-      </c>
-      <c r="G77" s="6" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H77" s="6" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="I77" t="n">
-        <v>-123</v>
-      </c>
-      <c r="J77" t="inlineStr">
-        <is>
-          <t>0/4</t>
-        </is>
-      </c>
-      <c r="K77" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L77" t="inlineStr"/>
-      <c r="M77" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>CIN@BAL</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>Joe Burrow</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>rush_yds</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>UNDER</t>
-        </is>
-      </c>
-      <c r="F78" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="G78" s="6" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H78" s="6" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="I78" t="n">
-        <v>-123</v>
-      </c>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t>2/5</t>
-        </is>
-      </c>
-      <c r="K78" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L78" t="inlineStr"/>
-      <c r="M78" t="inlineStr">
-        <is>
-          <t>opp QB: BAL fill-in QB (QB1 Out)</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>LEAN</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>CLE@TEN</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>Cam Ward</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>pass_att</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>OVER</t>
-        </is>
-      </c>
-      <c r="F79" t="n">
-        <v>30.5</v>
-      </c>
-      <c r="G79" s="6" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H79" s="6" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="I79" t="n">
-        <v>-122</v>
-      </c>
-      <c r="J79" t="inlineStr">
-        <is>
-          <t>4/6</t>
-        </is>
-      </c>
-      <c r="K79" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L79" t="inlineStr"/>
-      <c r="M79" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>